<commit_message>
Align Dermolab solution with the professor's slides
Interest split 20k/10k, depreciation 31k + 31k, own work at 30/h,
full-year amortization 142k and impairment 278k; explain P&L credits.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012nWMFk2orvaisxGrBVUj46
</commit_message>
<xml_diff>
--- a/Accounting/Dermolab_solution.xlsx
+++ b/Accounting/Dermolab_solution.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="339">
   <si>
     <t xml:space="preserve">FINANCIAL ACCOUNTING HOMEWORK TEMPLATE</t>
   </si>
@@ -368,7 +368,7 @@
     <t xml:space="preserve">Land donated by Viladecans (promised Jul 2018, formalized Jan 2019)</t>
   </si>
   <si>
-    <t xml:space="preserve">Jan 2019: asset LAND at fair value; credit deferred income (grant). No entry in 2018.</t>
+    <t xml:space="preserve">Jan 2019: asset LAND at fair value; credit Grant/Donation as a LIABILITY. No entry in 2018. Land is not depreciated, so the grant is not released to the P&amp;L (slide 2).</t>
   </si>
   <si>
     <t xml:space="preserve">A conditional promise isn't an asset until the condition (jobs) is met (IAS 20.7). A non-monetary grant is measured at FAIR VALUE (750,000, the expert appraisal); the 550,000 is only a tax value.</t>
@@ -404,10 +404,10 @@
     <t xml:space="preserve">New building &amp; production facilities (2019, in use Jan 2020)</t>
   </si>
   <si>
-    <t xml:space="preserve">During 2019: construction in progress (not depreciated). Jan 2020: transfer to Buildings 630,000 and Facilities 300,000.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All costs to bring the asset into use are capitalized: building 450,000 + management &amp; permits 150,000; facilities 240,000 + installation 60,000. 2019 loan interest (30,000) is CAPITALIZED, because a building taking a year to construct is a qualifying asset (IAS 23). From 2020 interest is an expense. Depreciation: building 630,000 / 20 = 31,500/yr; facilities 300,000 / 10 = 30,000/yr.</t>
+    <t xml:space="preserve">During 2019: construction in progress (not depreciated). Jan 2020: transfer to Buildings 620,000 and Facilities 310,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All costs to bring the asset into use are capitalized: building 450,000 + management &amp; permits 150,000; facilities 240,000 + installation 60,000. 2019 loan interest (30,000) is CAPITALIZED (IAS 23) and split by cost: 20,000 building (600/900) + 10,000 facilities (300/900). From 2020 interest is an expense (570,000 × 5% = 28,500). Depreciation: building 620,000 / 20 = 31,000/yr; facilities 310,000 / 10 = 31,000/yr.</t>
   </si>
   <si>
     <t xml:space="preserve">5</t>
@@ -440,10 +440,10 @@
     <t xml:space="preserve">New equipment bought in 2020</t>
   </si>
   <si>
-    <t xml:space="preserve">Cost = 200,000 − 2% (4,000) + 600 transport + own installation 100 h × 20 = 198,600.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Purchase price NET of discounts plus every cost to bring it to working condition (IAS 16.16-17). Own staff at COST (20/h), recorded as 'own work capitalized' because the salaries are already expensed.</t>
+    <t xml:space="preserve">Cost = 200,000 − 2% (4,000) + 600 transport + own installation 100 h × (20 + 10) = 199,600.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purchase price NET of discounts plus every cost to bring it to working condition (IAS 16.16-17). Own staff at PRODUCTION COST: direct 20/h + reasonable overhead 10/h, never the 15/h profit. Credit P&amp;L 'own work capitalized' because the salaries are already expensed.</t>
   </si>
   <si>
     <t xml:space="preserve">8</t>
@@ -452,10 +452,10 @@
     <t xml:space="preserve">Patent bought (Jan 2021) + development (10,000 h × 42)</t>
   </si>
   <si>
-    <t xml:space="preserve">Patent 1,000,000 and development 420,000 → INTANGIBLE ASSETS. Amortize over 10 years starting NOVEMBER 2021.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acquired patent = intangible at cost (IAS 38.25). Development is capitalized when technically feasible, approved and marketable (IAS 38.57). Use the ECONOMIC life (10) when it is shorter than the legal life (15). Amortization starts when the asset is available for use (IAS 38.97): 1,420,000 / 10 × 2/12 = 23,667.</t>
+    <t xml:space="preserve">Patent 1,000,000 and development 420,000 → INTANGIBLE ASSETS (1,420,000). Amortize over 10 years: 142,000 for 2021.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acquired patent = intangible at cost (IAS 38.25). Development is capitalized when technically feasible, approved and marketable (IAS 38.57). Use the ECONOMIC life (10) when it is shorter than the legal life (15). The slides charge a full year: 1,420,000 / 10 = 142,000.</t>
   </si>
   <si>
     <t xml:space="preserve">9</t>
@@ -488,10 +488,10 @@
     <t xml:space="preserve">Competitor launches a substitute (Dec 2021)</t>
   </si>
   <si>
-    <t xml:space="preserve">IMPAIRMENT LOSS 396,333 to P&amp;L. From 2022, amortize the new 1,000,000 over 5 years (200,000/yr).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Book value 1,420,000 − 23,667 = 1,396,333. Recoverable amount = HIGHER of value in use (1,000,000) and fair value less costs to sell (800,000 offer) = 1,000,000 (IAS 36.18). Loss = 396,333. The 1,800,000 old estimate is irrelevant: an intangible is never written UP above cost.</t>
+    <t xml:space="preserve">IMPAIRMENT LOSS 278,000 to P&amp;L. From 2022, amortize the new 1,000,000 over 5 years (200,000/yr).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Book value 1,420,000 − 142,000 = 1,278,000. Recoverable amount = HIGHER of value in use (1,000,000) and fair value less costs to sell (800,000 offer) = 1,000,000 (IAS 36.18). Loss = 278,000. The 1,800,000 old estimate is irrelevant: an intangible is never written UP above cost.</t>
   </si>
   <si>
     <t xml:space="preserve">P&amp;L IMPACT BY YEAR (from these events only)</t>
@@ -539,28 +539,40 @@
     <t xml:space="preserve">2018 / 2019 column: everything is 2018 (the gain). 2019 has no P&amp;L effect: the interest is capitalized and the grant is deferred. Salaries of researchers/installers are not shown; they were already recorded as personnel expense.</t>
   </si>
   <si>
-    <t xml:space="preserve">ASSUMPTIONS &amp; POINTS TO CONFIRM WITH THE PROFESSOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Land donation (1): credited to DEFERRED INCOME (IAS 20). Alternatives you may see: credit straight to income in 2019 (the only condition, the jobs, was met), or to equity 'Donations received' (Spanish GAAP). The asset side, land at 750,000, is the same in all three.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Demolition (3): capitalized in the LAND. Some textbooks add it to the new building instead, which would mean depreciating it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Loan (4): instalments of 30,000 principal + interest paid each December, starting Dec 2019. All 2019 interest is capitalized in the building (the qualifying asset).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Facilities (4) come into use with the building in January 2020. The improvement (6) is done at end-2020 and depreciated over 10 years from 2021.</t>
+    <t xml:space="preserve">WHY IS THE P&amp;L CREDITED IN EVENTS 7 AND 8? (and why it is DEBITED in 11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• The rule hasn't changed: an expense is a DEBIT to the P&amp;L. In events 7 and 8 the expense was ALREADY debited, when the staff were paid during the year: Dr P&amp;L – Salaries / Cr Cash.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Some of those salaries were not a cost of running the business: they created an asset (the installed equipment in 7, the Baldnessox development in 8). That part must leave the P&amp;L and go into the asset.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• To take a debit out of the P&amp;L you CREDIT it: Dr Development costs (asset) 420,000 / Cr P&amp;L 420,000. The net result: salaries 420,000 debit − 420,000 credit = 0 in the P&amp;L, and the asset holds 420,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Spanish GAAP (by nature) shows the credit as an income line, 'Work carried out by the company for its own assets'. IFRS (by function) shows it as a reduction of salaries ('Salaries &amp; other expenses − 3,000'). Same entry, two presentations (slide 11).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• The asset is then expensed LATER, through amortization (event 11: 142,000 a year), so the cost reaches the P&amp;L in the years when the product earns revenue.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Event 11 is the opposite: amortization 142,000 and impairment 278,000 are real losses of value, so the P&amp;L is DEBITED. The CREDITS go to Accumulated amortization and Accumulated impairment, which are contra-assets that reduce the patent's book value to 1,000,000 (slide 36).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSUMPTIONS (where the case is silent; the slides settle the rest)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Loan (4): 30,000 of principal (600,000 / 20) plus interest paid each December, starting Dec 2019. Slide 8 says 'Loan: 1 Jan 2020', but the case says January 2019, and the capitalized 2019 interest only works with 2019.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Facilities (4) come into use with the building in January 2020. The improvement (6) is depreciated over 10 years from 2021 (4,000/yr, slide 10).</t>
   </si>
   <si>
     <t xml:space="preserve">• New equipment (7): no useful life is given, so no depreciation is computed.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Research hours (9) are valued at the same 42/h as the development hours (8); they matter only as an explanation, because they are already in salaries.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Old premises (2): their cost and accumulated depreciation are entered as beginning balances (BB) in the T-accounts, because only the sale is recorded here. The cash T-account starts at zero, so its ending balance is not the real bank balance.</t>
+    <t xml:space="preserve">• Old premises (2): their cost and accumulated depreciation are entered as beginning balances (BB), because only the sale is recorded here. The cash T-account starts at zero, so its ending balance is not the real bank balance.</t>
   </si>
   <si>
     <t xml:space="preserve">JOURNAL ENTRIES</t>
@@ -701,7 +713,7 @@
     <t xml:space="preserve">4c</t>
   </si>
   <si>
-    <t xml:space="preserve">Dec 2019 – interest 600,000 × 5% CAPITALIZED (asset under construction)</t>
+    <t xml:space="preserve">Dec 2019 – interest 600,000 × 5% CAPITALIZED: 20,000 building + 10,000 facilities (2/3 – 1/3 of cost)</t>
   </si>
   <si>
     <t xml:space="preserve">O</t>
@@ -719,7 +731,7 @@
     <t xml:space="preserve">4e</t>
   </si>
   <si>
-    <t xml:space="preserve">Jan 2020 – construction finished: building 600,000 + 30,000 interest; facilities 300,000</t>
+    <t xml:space="preserve">Jan 2020 – construction finished: building 450 + 150 + 20 interest = 620,000; facilities 240 + 60 + 10 interest = 310,000</t>
   </si>
   <si>
     <t xml:space="preserve">Machinery &amp; production facilities</t>
@@ -746,7 +758,10 @@
     <t xml:space="preserve">7b</t>
   </si>
   <si>
-    <t xml:space="preserve">2020 – installation by own staff 100 h × 20 (cost, never the 45 price)</t>
+    <t xml:space="preserve">2020 – installation by own staff 100 h × (20 direct + 10 overhead) = 3,000; never the 15 profit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salaries were already expensed → move 3,000 out of the P&amp;L into the asset</t>
   </si>
   <si>
     <t xml:space="preserve">P&amp;L – Own work capitalized</t>
@@ -770,7 +785,7 @@
     <t xml:space="preserve">4h</t>
   </si>
   <si>
-    <t xml:space="preserve">Dec 2020 – depreciation: building 630,000 / 20; facilities 300,000 / 10</t>
+    <t xml:space="preserve">Dec 2020 – depreciation: building 620,000 / 20 = 31,000; facilities 310,000 / 10 = 31,000</t>
   </si>
   <si>
     <t xml:space="preserve">P&amp;L – Depreciation expense</t>
@@ -800,6 +815,9 @@
     <t xml:space="preserve">Development costs – Baldnessox</t>
   </si>
   <si>
+    <t xml:space="preserve">Salaries were already expensed → move 420,000 out of the P&amp;L into the asset</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jul–Dec 2021 – RESEARCH: external 224,000 → EXPENSE (17,000 h already in salaries)</t>
   </si>
   <si>
@@ -827,13 +845,13 @@
     <t xml:space="preserve">4k</t>
   </si>
   <si>
-    <t xml:space="preserve">Dec 2021 – depreciation: building 31,500; facilities 30,000 + improvement 40,000 / 10</t>
+    <t xml:space="preserve">Dec 2021 – depreciation: building 31,000; facilities 31,000 + improvement 40,000 / 10 = 4,000</t>
   </si>
   <si>
     <t xml:space="preserve">8c</t>
   </si>
   <si>
-    <t xml:space="preserve">Dec 2021 – amortization from NOVEMBER (in use): 1,420,000 / 10 × 2/12</t>
+    <t xml:space="preserve">Dec 2021 – amortization, full year: 1,420,000 / 10 = 142,000</t>
   </si>
   <si>
     <t xml:space="preserve">P&amp;L – Amortization expense</t>
@@ -842,7 +860,7 @@
     <t xml:space="preserve">Accum. amortization &amp; impairment – intangibles</t>
   </si>
   <si>
-    <t xml:space="preserve">Dec 2021 – impairment: book 1,396,333 vs recoverable 1,000,000 (higher of 1,000,000 VIU and 800,000 offer)</t>
+    <t xml:space="preserve">Dec 2021 – impairment: book 1,278,000 vs recoverable 1,000,000 (higher of 1,000,000 VIU and 800,000 offer)</t>
   </si>
   <si>
     <t xml:space="preserve">P&amp;L – Impairment loss</t>
@@ -2776,7 +2794,7 @@
     <tabColor rgb="FFC00000"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:F36"/>
+  <dimension ref="B1:F41"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2930,7 +2948,7 @@
         <v>139</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>198600</v>
+        <v>199600</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2998,7 +3016,7 @@
         <v>155</v>
       </c>
       <c r="F14" s="33" t="n">
-        <v>396333</v>
+        <v>278000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3060,7 +3078,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="37" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="F20" s="37" t="n">
         <v>420000</v>
@@ -3102,10 +3120,10 @@
         <v>0</v>
       </c>
       <c r="E23" s="37" t="n">
-        <v>-61500</v>
+        <v>-62000</v>
       </c>
       <c r="F23" s="37" t="n">
-        <v>-65500</v>
+        <v>-66000</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3119,7 +3137,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="37" t="n">
-        <v>-23667</v>
+        <v>-142000</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3133,7 +3151,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="37" t="n">
-        <v>-396333</v>
+        <v>-278000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3146,11 +3164,11 @@
       </c>
       <c r="E26" s="39" t="n">
         <f aca="false">SUM(E18:E25)</f>
-        <v>-96000</v>
+        <v>-95500</v>
       </c>
       <c r="F26" s="39" t="n">
         <f aca="false">SUM(F18:F25)</f>
-        <v>-316500</v>
+        <v>-317000</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3225,17 +3243,53 @@
       <c r="E35" s="40"/>
       <c r="F35" s="40"/>
     </row>
-    <row r="36" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="40" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="34" t="s">
         <v>178</v>
       </c>
-      <c r="C36" s="40"/>
-      <c r="D36" s="40"/>
-      <c r="E36" s="40"/>
-      <c r="F36" s="40"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="34"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="34"/>
+    </row>
+    <row r="38" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="C38" s="40"/>
+      <c r="D38" s="40"/>
+      <c r="E38" s="40"/>
+      <c r="F38" s="40"/>
+    </row>
+    <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="40" t="s">
+        <v>180</v>
+      </c>
+      <c r="C39" s="40"/>
+      <c r="D39" s="40"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="40"/>
+    </row>
+    <row r="40" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B40" s="40" t="s">
+        <v>181</v>
+      </c>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
+    </row>
+    <row r="41" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B41" s="40" t="s">
+        <v>182</v>
+      </c>
+      <c r="C41" s="40"/>
+      <c r="D41" s="40"/>
+      <c r="E41" s="40"/>
+      <c r="F41" s="40"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="15">
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B27:F27"/>
@@ -3246,7 +3300,11 @@
     <mergeCell ref="B33:F33"/>
     <mergeCell ref="B34:F34"/>
     <mergeCell ref="B35:F35"/>
-    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="B41:F41"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3279,7 +3337,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -3291,7 +3349,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="3" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C2" s="41" t="str">
         <f aca="false">Guide!$C$3</f>
@@ -3299,7 +3357,7 @@
       </c>
       <c r="D2" s="41"/>
       <c r="E2" s="3" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="F2" s="41" t="str">
         <f aca="false">Guide!$C$4</f>
@@ -3309,15 +3367,15 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C4" s="42" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="E4" s="43" t="n">
         <f aca="false">SUM(E7:E106)</f>
-        <v>24318100</v>
+        <v>24320100</v>
       </c>
       <c r="F4" s="43" t="n">
         <f aca="false">SUM(F7:F106)</f>
-        <v>24318100</v>
+        <v>24320100</v>
       </c>
       <c r="G4" s="44" t="str">
         <f aca="false">IF(ABS(E4-F4)&lt;0.5,"OK","ERROR: "&amp;TEXT(E4-F4,"#,##0"))</f>
@@ -3330,10 +3388,10 @@
         <v>107</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D6" s="45" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E6" s="45" t="s">
         <v>64</v>
@@ -3345,13 +3403,13 @@
         <v>66</v>
       </c>
       <c r="H6" s="45" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="I6" s="45" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="K6" s="46" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3359,10 +3417,10 @@
         <v>112</v>
       </c>
       <c r="C7" s="48" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D7" s="48" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="E7" s="49"/>
       <c r="F7" s="49"/>
@@ -3373,7 +3431,7 @@
         <v>OK</v>
       </c>
       <c r="K7" s="51" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3381,10 +3439,10 @@
         <v>116</v>
       </c>
       <c r="C8" s="53" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D8" s="53" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E8" s="54" t="n">
         <v>13000000</v>
@@ -3394,14 +3452,14 @@
         <v>69</v>
       </c>
       <c r="H8" s="52" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="I8" s="50" t="str">
         <f aca="false">IF(B8="","",IF(ABS(SUMIF($B$7:$B$106,B8,$E$7:$E$106)-SUMIF($B$7:$B$106,B8,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
         <v>OK</v>
       </c>
       <c r="K8" s="55" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3410,14 +3468,14 @@
       </c>
       <c r="C9" s="48"/>
       <c r="D9" s="48" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="E9" s="49" t="n">
         <v>5400000</v>
       </c>
       <c r="F9" s="49"/>
       <c r="G9" s="47" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="H9" s="47"/>
       <c r="I9" s="50" t="str">
@@ -3425,7 +3483,7 @@
         <v>OK</v>
       </c>
       <c r="K9" s="55" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3434,14 +3492,14 @@
       </c>
       <c r="C10" s="53"/>
       <c r="D10" s="53" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E10" s="54"/>
       <c r="F10" s="54" t="n">
         <v>5000000</v>
       </c>
       <c r="G10" s="52" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H10" s="52"/>
       <c r="I10" s="50" t="str">
@@ -3449,7 +3507,7 @@
         <v>OK</v>
       </c>
       <c r="K10" s="55" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3458,14 +3516,14 @@
       </c>
       <c r="C11" s="48"/>
       <c r="D11" s="48" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="E11" s="49"/>
       <c r="F11" s="49" t="n">
         <v>6000000</v>
       </c>
       <c r="G11" s="47" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H11" s="47"/>
       <c r="I11" s="50" t="str">
@@ -3473,7 +3531,7 @@
         <v>OK</v>
       </c>
       <c r="K11" s="55" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3481,17 +3539,17 @@
         <v>116</v>
       </c>
       <c r="C12" s="53" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D12" s="53" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E12" s="54"/>
       <c r="F12" s="54" t="n">
         <v>7400000</v>
       </c>
       <c r="G12" s="52" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="H12" s="52"/>
       <c r="I12" s="50" t="str">
@@ -3499,7 +3557,7 @@
         <v>OK</v>
       </c>
       <c r="K12" s="55" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3507,10 +3565,10 @@
         <v>112</v>
       </c>
       <c r="C13" s="48" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D13" s="48" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E13" s="49" t="n">
         <v>750000</v>
@@ -3520,14 +3578,14 @@
         <v>69</v>
       </c>
       <c r="H13" s="47" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="I13" s="50" t="str">
         <f aca="false">IF(B13="","",IF(ABS(SUMIF($B$7:$B$106,B13,$E$7:$E$106)-SUMIF($B$7:$B$106,B13,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
         <v>OK</v>
       </c>
       <c r="K13" s="55" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3536,7 +3594,7 @@
       </c>
       <c r="C14" s="53"/>
       <c r="D14" s="53" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="E14" s="54"/>
       <c r="F14" s="54" t="n">
@@ -3551,7 +3609,7 @@
         <v>OK</v>
       </c>
       <c r="K14" s="51" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3559,10 +3617,10 @@
         <v>120</v>
       </c>
       <c r="C15" s="48" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="D15" s="48" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E15" s="49" t="n">
         <v>125000</v>
@@ -3577,7 +3635,7 @@
         <v>OK</v>
       </c>
       <c r="K15" s="55" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3586,35 +3644,35 @@
       </c>
       <c r="C16" s="53"/>
       <c r="D16" s="53" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E16" s="54"/>
       <c r="F16" s="54" t="n">
         <v>125000</v>
       </c>
       <c r="G16" s="52" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H16" s="52" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="I16" s="50" t="str">
         <f aca="false">IF(B16="","",IF(ABS(SUMIF($B$7:$B$106,B16,$E$7:$E$106)-SUMIF($B$7:$B$106,B16,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
         <v>OK</v>
       </c>
       <c r="K16" s="55" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="47" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C17" s="48" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="D17" s="48" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E17" s="49" t="n">
         <v>600000</v>
@@ -3624,23 +3682,23 @@
         <v>69</v>
       </c>
       <c r="H17" s="47" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="I17" s="50" t="str">
         <f aca="false">IF(B17="","",IF(ABS(SUMIF($B$7:$B$106,B17,$E$7:$E$106)-SUMIF($B$7:$B$106,B17,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
         <v>OK</v>
       </c>
       <c r="K17" s="51" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="52" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C18" s="53"/>
       <c r="D18" s="53" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E18" s="54"/>
       <c r="F18" s="54" t="n">
@@ -3655,18 +3713,18 @@
         <v>OK</v>
       </c>
       <c r="K18" s="55" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="47" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C19" s="48" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D19" s="48" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E19" s="49" t="n">
         <v>900000</v>
@@ -3683,21 +3741,21 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="52" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C20" s="53"/>
       <c r="D20" s="53" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E20" s="54"/>
       <c r="F20" s="54" t="n">
         <v>900000</v>
       </c>
       <c r="G20" s="52" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H20" s="52" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="I20" s="50" t="str">
         <f aca="false">IF(B20="","",IF(ABS(SUMIF($B$7:$B$106,B20,$E$7:$E$106)-SUMIF($B$7:$B$106,B20,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -3706,13 +3764,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="47" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C21" s="48" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="D21" s="48" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E21" s="49" t="n">
         <v>30000</v>
@@ -3729,21 +3787,21 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="52" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C22" s="53"/>
       <c r="D22" s="53" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E22" s="54"/>
       <c r="F22" s="54" t="n">
         <v>30000</v>
       </c>
       <c r="G22" s="52" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H22" s="52" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="I22" s="50" t="str">
         <f aca="false">IF(B22="","",IF(ABS(SUMIF($B$7:$B$106,B22,$E$7:$E$106)-SUMIF($B$7:$B$106,B22,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -3752,20 +3810,20 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="47" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C23" s="48" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="D23" s="48" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E23" s="49" t="n">
         <v>30000</v>
       </c>
       <c r="F23" s="49"/>
       <c r="G23" s="47" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="H23" s="47"/>
       <c r="I23" s="50" t="str">
@@ -3775,21 +3833,21 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="52" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C24" s="53"/>
       <c r="D24" s="53" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E24" s="54"/>
       <c r="F24" s="54" t="n">
         <v>30000</v>
       </c>
       <c r="G24" s="52" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H24" s="52" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="I24" s="50" t="str">
         <f aca="false">IF(B24="","",IF(ABS(SUMIF($B$7:$B$106,B24,$E$7:$E$106)-SUMIF($B$7:$B$106,B24,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -3798,23 +3856,23 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="47" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C25" s="48" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="D25" s="48" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="E25" s="49" t="n">
-        <v>630000</v>
+        <v>620000</v>
       </c>
       <c r="F25" s="49"/>
       <c r="G25" s="47" t="s">
         <v>69</v>
       </c>
       <c r="H25" s="47" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="I25" s="50" t="str">
         <f aca="false">IF(B25="","",IF(ABS(SUMIF($B$7:$B$106,B25,$E$7:$E$106)-SUMIF($B$7:$B$106,B25,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -3823,14 +3881,14 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="52" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C26" s="53"/>
       <c r="D26" s="53" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E26" s="54" t="n">
-        <v>300000</v>
+        <v>310000</v>
       </c>
       <c r="F26" s="54"/>
       <c r="G26" s="52" t="s">
@@ -3844,18 +3902,18 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="47" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C27" s="48"/>
       <c r="D27" s="48" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E27" s="49"/>
       <c r="F27" s="49" t="n">
         <v>930000</v>
       </c>
       <c r="G27" s="47" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H27" s="47"/>
       <c r="I27" s="50" t="str">
@@ -3868,17 +3926,17 @@
         <v>128</v>
       </c>
       <c r="C28" s="53" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D28" s="53" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E28" s="54" t="n">
         <v>8000</v>
       </c>
       <c r="F28" s="54"/>
       <c r="G28" s="52" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H28" s="52"/>
       <c r="I28" s="50" t="str">
@@ -3892,17 +3950,17 @@
       </c>
       <c r="C29" s="48"/>
       <c r="D29" s="48" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E29" s="49"/>
       <c r="F29" s="49" t="n">
         <v>8000</v>
       </c>
       <c r="G29" s="47" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H29" s="47" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="I29" s="50" t="str">
         <f aca="false">IF(B29="","",IF(ABS(SUMIF($B$7:$B$106,B29,$E$7:$E$106)-SUMIF($B$7:$B$106,B29,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -3914,10 +3972,10 @@
         <v>132</v>
       </c>
       <c r="C30" s="53" t="s">
+        <v>240</v>
+      </c>
+      <c r="D30" s="53" t="s">
         <v>236</v>
-      </c>
-      <c r="D30" s="53" t="s">
-        <v>232</v>
       </c>
       <c r="E30" s="54" t="n">
         <v>40000</v>
@@ -3938,17 +3996,17 @@
       </c>
       <c r="C31" s="48"/>
       <c r="D31" s="48" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E31" s="49"/>
       <c r="F31" s="49" t="n">
         <v>40000</v>
       </c>
       <c r="G31" s="47" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H31" s="47" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="I31" s="50" t="str">
         <f aca="false">IF(B31="","",IF(ABS(SUMIF($B$7:$B$106,B31,$E$7:$E$106)-SUMIF($B$7:$B$106,B31,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -3957,13 +4015,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="52" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C32" s="53" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D32" s="53" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E32" s="54" t="n">
         <v>196600</v>
@@ -3980,21 +4038,21 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="47" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C33" s="48"/>
       <c r="D33" s="48" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E33" s="49"/>
       <c r="F33" s="49" t="n">
         <v>196600</v>
       </c>
       <c r="G33" s="47" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H33" s="47" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="I33" s="50" t="str">
         <f aca="false">IF(B33="","",IF(ABS(SUMIF($B$7:$B$106,B33,$E$7:$E$106)-SUMIF($B$7:$B$106,B33,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4003,23 +4061,23 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="52" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C34" s="53" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D34" s="53" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E34" s="54" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="F34" s="54"/>
       <c r="G34" s="52" t="s">
         <v>69</v>
       </c>
       <c r="H34" s="52" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="I34" s="50" t="str">
         <f aca="false">IF(B34="","",IF(ABS(SUMIF($B$7:$B$106,B34,$E$7:$E$106)-SUMIF($B$7:$B$106,B34,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4028,18 +4086,20 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="47" t="s">
-        <v>239</v>
-      </c>
-      <c r="C35" s="48"/>
+        <v>243</v>
+      </c>
+      <c r="C35" s="48" t="s">
+        <v>245</v>
+      </c>
       <c r="D35" s="48" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E35" s="49"/>
       <c r="F35" s="49" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G35" s="47" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="H35" s="47"/>
       <c r="I35" s="50" t="str">
@@ -4049,20 +4109,20 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="52" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="C36" s="53" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="D36" s="53" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="E36" s="54" t="n">
         <v>28500</v>
       </c>
       <c r="F36" s="54"/>
       <c r="G36" s="52" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H36" s="52"/>
       <c r="I36" s="50" t="str">
@@ -4072,21 +4132,21 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="47" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="C37" s="48"/>
       <c r="D37" s="48" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E37" s="49"/>
       <c r="F37" s="49" t="n">
         <v>28500</v>
       </c>
       <c r="G37" s="47" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H37" s="47" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="I37" s="50" t="str">
         <f aca="false">IF(B37="","",IF(ABS(SUMIF($B$7:$B$106,B37,$E$7:$E$106)-SUMIF($B$7:$B$106,B37,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4095,20 +4155,20 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="52" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C38" s="53" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D38" s="53" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E38" s="54" t="n">
         <v>30000</v>
       </c>
       <c r="F38" s="54"/>
       <c r="G38" s="52" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="H38" s="52"/>
       <c r="I38" s="50" t="str">
@@ -4118,21 +4178,21 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="47" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C39" s="48"/>
       <c r="D39" s="48" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E39" s="49"/>
       <c r="F39" s="49" t="n">
         <v>30000</v>
       </c>
       <c r="G39" s="47" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H39" s="47" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="I39" s="50" t="str">
         <f aca="false">IF(B39="","",IF(ABS(SUMIF($B$7:$B$106,B39,$E$7:$E$106)-SUMIF($B$7:$B$106,B39,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4141,23 +4201,23 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="52" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C40" s="53" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="D40" s="53" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="E40" s="54" t="n">
-        <v>61500</v>
+        <v>62000</v>
       </c>
       <c r="F40" s="54"/>
       <c r="G40" s="52" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H40" s="52" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="I40" s="50" t="str">
         <f aca="false">IF(B40="","",IF(ABS(SUMIF($B$7:$B$106,B40,$E$7:$E$106)-SUMIF($B$7:$B$106,B40,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4166,18 +4226,18 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="47" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C41" s="48"/>
       <c r="D41" s="48" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="E41" s="49"/>
       <c r="F41" s="49" t="n">
-        <v>31500</v>
+        <v>31000</v>
       </c>
       <c r="G41" s="47" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="H41" s="47"/>
       <c r="I41" s="50" t="str">
@@ -4187,18 +4247,18 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="52" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C42" s="53"/>
       <c r="D42" s="53" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E42" s="54"/>
       <c r="F42" s="54" t="n">
-        <v>30000</v>
+        <v>31000</v>
       </c>
       <c r="G42" s="52" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="H42" s="52"/>
       <c r="I42" s="50" t="str">
@@ -4208,13 +4268,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="47" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C43" s="48" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D43" s="48" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="E43" s="49" t="n">
         <v>1000000</v>
@@ -4231,21 +4291,21 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="52" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C44" s="53"/>
       <c r="D44" s="53" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E44" s="54"/>
       <c r="F44" s="54" t="n">
         <v>1000000</v>
       </c>
       <c r="G44" s="52" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H44" s="52" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="I44" s="50" t="str">
         <f aca="false">IF(B44="","",IF(ABS(SUMIF($B$7:$B$106,B44,$E$7:$E$106)-SUMIF($B$7:$B$106,B44,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4254,13 +4314,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="47" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C45" s="48" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D45" s="48" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E45" s="49" t="n">
         <v>420000</v>
@@ -4270,7 +4330,7 @@
         <v>69</v>
       </c>
       <c r="H45" s="47" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="I45" s="50" t="str">
         <f aca="false">IF(B45="","",IF(ABS(SUMIF($B$7:$B$106,B45,$E$7:$E$106)-SUMIF($B$7:$B$106,B45,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4279,18 +4339,20 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="52" t="s">
-        <v>255</v>
-      </c>
-      <c r="C46" s="53"/>
+        <v>260</v>
+      </c>
+      <c r="C46" s="53" t="s">
+        <v>263</v>
+      </c>
       <c r="D46" s="53" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E46" s="54"/>
       <c r="F46" s="54" t="n">
         <v>420000</v>
       </c>
       <c r="G46" s="52" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="H46" s="52"/>
       <c r="I46" s="50" t="str">
@@ -4303,17 +4365,17 @@
         <v>144</v>
       </c>
       <c r="C47" s="48" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="D47" s="48" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="E47" s="49" t="n">
         <v>224000</v>
       </c>
       <c r="F47" s="49"/>
       <c r="G47" s="47" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H47" s="47"/>
       <c r="I47" s="50" t="str">
@@ -4327,17 +4389,17 @@
       </c>
       <c r="C48" s="53"/>
       <c r="D48" s="53" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E48" s="54"/>
       <c r="F48" s="54" t="n">
         <v>224000</v>
       </c>
       <c r="G48" s="52" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H48" s="52" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="I48" s="50" t="str">
         <f aca="false">IF(B48="","",IF(ABS(SUMIF($B$7:$B$106,B48,$E$7:$E$106)-SUMIF($B$7:$B$106,B48,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4349,10 +4411,10 @@
         <v>148</v>
       </c>
       <c r="C49" s="48" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="D49" s="48" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="E49" s="49"/>
       <c r="F49" s="49"/>
@@ -4365,20 +4427,20 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="52" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="C50" s="53" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="D50" s="53" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="E50" s="54" t="n">
         <v>27000</v>
       </c>
       <c r="F50" s="54"/>
       <c r="G50" s="52" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H50" s="52"/>
       <c r="I50" s="50" t="str">
@@ -4388,21 +4450,21 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="47" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="C51" s="48"/>
       <c r="D51" s="48" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E51" s="49"/>
       <c r="F51" s="49" t="n">
         <v>27000</v>
       </c>
       <c r="G51" s="47" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H51" s="47" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="I51" s="50" t="str">
         <f aca="false">IF(B51="","",IF(ABS(SUMIF($B$7:$B$106,B51,$E$7:$E$106)-SUMIF($B$7:$B$106,B51,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4411,20 +4473,20 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="52" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="C52" s="53" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="D52" s="53" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E52" s="54" t="n">
         <v>30000</v>
       </c>
       <c r="F52" s="54"/>
       <c r="G52" s="52" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="H52" s="52"/>
       <c r="I52" s="50" t="str">
@@ -4434,21 +4496,21 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="47" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="C53" s="48"/>
       <c r="D53" s="48" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E53" s="49"/>
       <c r="F53" s="49" t="n">
         <v>30000</v>
       </c>
       <c r="G53" s="47" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H53" s="47" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="I53" s="50" t="str">
         <f aca="false">IF(B53="","",IF(ABS(SUMIF($B$7:$B$106,B53,$E$7:$E$106)-SUMIF($B$7:$B$106,B53,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4457,23 +4519,23 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="52" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="C54" s="53" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="D54" s="53" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="E54" s="54" t="n">
-        <v>65500</v>
+        <v>66000</v>
       </c>
       <c r="F54" s="54"/>
       <c r="G54" s="52" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H54" s="52" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="I54" s="50" t="str">
         <f aca="false">IF(B54="","",IF(ABS(SUMIF($B$7:$B$106,B54,$E$7:$E$106)-SUMIF($B$7:$B$106,B54,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4482,18 +4544,18 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="47" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="C55" s="48"/>
       <c r="D55" s="48" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="E55" s="49"/>
       <c r="F55" s="49" t="n">
-        <v>31500</v>
+        <v>31000</v>
       </c>
       <c r="G55" s="47" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="H55" s="47"/>
       <c r="I55" s="50" t="str">
@@ -4503,18 +4565,18 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="52" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="C56" s="53"/>
       <c r="D56" s="53" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E56" s="54"/>
       <c r="F56" s="54" t="n">
-        <v>34000</v>
+        <v>35000</v>
       </c>
       <c r="G56" s="52" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="H56" s="52"/>
       <c r="I56" s="50" t="str">
@@ -4524,23 +4586,23 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="47" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="C57" s="48" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D57" s="48" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="E57" s="49" t="n">
-        <v>23667</v>
+        <v>142000</v>
       </c>
       <c r="F57" s="49"/>
       <c r="G57" s="47" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H57" s="47" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="I57" s="50" t="str">
         <f aca="false">IF(B57="","",IF(ABS(SUMIF($B$7:$B$106,B57,$E$7:$E$106)-SUMIF($B$7:$B$106,B57,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4549,18 +4611,18 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="52" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="C58" s="53"/>
       <c r="D58" s="53" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="E58" s="54"/>
       <c r="F58" s="54" t="n">
-        <v>23667</v>
+        <v>142000</v>
       </c>
       <c r="G58" s="52" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="H58" s="52"/>
       <c r="I58" s="50" t="str">
@@ -4573,20 +4635,20 @@
         <v>152</v>
       </c>
       <c r="C59" s="48" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="D59" s="48" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="E59" s="49" t="n">
-        <v>396333</v>
+        <v>278000</v>
       </c>
       <c r="F59" s="49"/>
       <c r="G59" s="47" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H59" s="47" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="I59" s="50" t="str">
         <f aca="false">IF(B59="","",IF(ABS(SUMIF($B$7:$B$106,B59,$E$7:$E$106)-SUMIF($B$7:$B$106,B59,$F$7:$F$106))&lt;0.5,"OK","ERROR: Dr≠Cr"))</f>
@@ -4599,14 +4661,14 @@
       </c>
       <c r="C60" s="53"/>
       <c r="D60" s="53" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="E60" s="54"/>
       <c r="F60" s="54" t="n">
-        <v>396333</v>
+        <v>278000</v>
       </c>
       <c r="G60" s="52" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="H60" s="52"/>
       <c r="I60" s="50" t="str">
@@ -5291,7 +5353,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="2" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -5314,7 +5376,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="3" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D2" s="41" t="str">
         <f aca="false">Guide!$C$3</f>
@@ -5326,7 +5388,7 @@
       <c r="H2" s="41"/>
       <c r="I2" s="41"/>
       <c r="L2" s="3" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="N2" s="41" t="str">
         <f aca="false">Guide!$C$4</f>
@@ -5339,7 +5401,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="56" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C5" s="56"/>
       <c r="D5" s="56"/>
@@ -5350,7 +5412,7 @@
       <c r="I5" s="56"/>
       <c r="J5" s="56"/>
       <c r="L5" s="57" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="M5" s="57"/>
       <c r="N5" s="57"/>
@@ -5361,41 +5423,41 @@
       <c r="S5" s="57"/>
       <c r="T5" s="57"/>
       <c r="W5" s="46" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="W6" s="51" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="58" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C7" s="58"/>
       <c r="D7" s="58"/>
       <c r="E7" s="58"/>
       <c r="G7" s="58" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="H7" s="58"/>
       <c r="I7" s="58"/>
       <c r="J7" s="58"/>
       <c r="M7" s="59" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="N7" s="59"/>
       <c r="O7" s="59"/>
       <c r="P7" s="59"/>
       <c r="R7" s="59" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="S7" s="59"/>
       <c r="T7" s="59"/>
       <c r="U7" s="59"/>
       <c r="W7" s="55" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5403,10 +5465,10 @@
         <v>107</v>
       </c>
       <c r="C8" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="D8" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E8" s="60" t="s">
         <v>107</v>
@@ -5415,10 +5477,10 @@
         <v>107</v>
       </c>
       <c r="H8" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="I8" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="J8" s="60" t="s">
         <v>107</v>
@@ -5427,10 +5489,10 @@
         <v>107</v>
       </c>
       <c r="N8" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="O8" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="P8" s="60" t="s">
         <v>107</v>
@@ -5439,27 +5501,27 @@
         <v>107</v>
       </c>
       <c r="S8" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="T8" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="U8" s="60" t="s">
         <v>107</v>
       </c>
       <c r="W8" s="55" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C9" s="63"/>
       <c r="D9" s="64"/>
       <c r="E9" s="62"/>
       <c r="G9" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="H9" s="63"/>
       <c r="I9" s="64"/>
@@ -5468,16 +5530,16 @@
       <c r="N9" s="63"/>
       <c r="O9" s="64"/>
       <c r="P9" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="R9" s="62"/>
       <c r="S9" s="63"/>
       <c r="T9" s="64"/>
       <c r="U9" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="W9" s="55" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5506,12 +5568,12 @@
       <c r="T10" s="54"/>
       <c r="U10" s="65"/>
       <c r="W10" s="51" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="65" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C11" s="66" t="n">
         <v>600000</v>
@@ -5520,7 +5582,7 @@
         <v>900000</v>
       </c>
       <c r="E11" s="65" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="G11" s="65"/>
       <c r="H11" s="66"/>
@@ -5535,7 +5597,7 @@
       <c r="T11" s="54"/>
       <c r="U11" s="65"/>
       <c r="W11" s="55" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5545,7 +5607,7 @@
         <v>30000</v>
       </c>
       <c r="E12" s="65" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G12" s="65"/>
       <c r="H12" s="66"/>
@@ -5560,7 +5622,7 @@
       <c r="T12" s="54"/>
       <c r="U12" s="65"/>
       <c r="W12" s="51" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5570,7 +5632,7 @@
         <v>30000</v>
       </c>
       <c r="E13" s="65" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="G13" s="65"/>
       <c r="H13" s="66"/>
@@ -5585,7 +5647,7 @@
       <c r="T13" s="54"/>
       <c r="U13" s="65"/>
       <c r="W13" s="55" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5610,7 +5672,7 @@
       <c r="T14" s="54"/>
       <c r="U14" s="65"/>
       <c r="W14" s="51" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5635,7 +5697,7 @@
       <c r="T15" s="54"/>
       <c r="U15" s="65"/>
       <c r="W15" s="55" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5645,7 +5707,7 @@
         <v>196600</v>
       </c>
       <c r="E16" s="65" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="G16" s="65"/>
       <c r="H16" s="66"/>
@@ -5660,7 +5722,7 @@
       <c r="T16" s="54"/>
       <c r="U16" s="65"/>
       <c r="W16" s="55" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5670,7 +5732,7 @@
         <v>28500</v>
       </c>
       <c r="E17" s="65" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="G17" s="65"/>
       <c r="H17" s="66"/>
@@ -5685,7 +5747,7 @@
       <c r="T17" s="54"/>
       <c r="U17" s="65"/>
       <c r="W17" s="51" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5695,7 +5757,7 @@
         <v>30000</v>
       </c>
       <c r="E18" s="65" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="G18" s="65"/>
       <c r="H18" s="66"/>
@@ -5710,7 +5772,7 @@
       <c r="T18" s="54"/>
       <c r="U18" s="65"/>
       <c r="W18" s="55" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5720,7 +5782,7 @@
         <v>1000000</v>
       </c>
       <c r="E19" s="65" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="G19" s="65"/>
       <c r="H19" s="66"/>
@@ -5735,7 +5797,7 @@
       <c r="T19" s="54"/>
       <c r="U19" s="65"/>
       <c r="W19" s="55" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5760,7 +5822,7 @@
       <c r="T20" s="54"/>
       <c r="U20" s="65"/>
       <c r="W20" s="51" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5770,7 +5832,7 @@
         <v>27000</v>
       </c>
       <c r="E21" s="65" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="G21" s="65"/>
       <c r="H21" s="66"/>
@@ -5785,7 +5847,7 @@
       <c r="T21" s="54"/>
       <c r="U21" s="65"/>
       <c r="W21" s="55" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5795,7 +5857,7 @@
         <v>30000</v>
       </c>
       <c r="E22" s="65" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G22" s="65"/>
       <c r="H22" s="66"/>
@@ -5810,7 +5872,7 @@
       <c r="T22" s="54"/>
       <c r="U22" s="65"/>
       <c r="W22" s="55" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5831,7 +5893,7 @@
       <c r="T23" s="54"/>
       <c r="U23" s="65"/>
       <c r="W23" s="55" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5852,12 +5914,12 @@
       <c r="T24" s="54"/>
       <c r="U24" s="65"/>
       <c r="W24" s="55" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C25" s="68" t="n">
         <f aca="false">SUM(C9:C24)</f>
@@ -5868,10 +5930,10 @@
         <v>2669100</v>
       </c>
       <c r="E25" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="G25" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="H25" s="68" t="n">
         <f aca="false">SUM(H9:H24)</f>
@@ -5882,10 +5944,10 @@
         <v>0</v>
       </c>
       <c r="J25" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="M25" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="N25" s="68" t="n">
         <f aca="false">SUM(N9:N24)</f>
@@ -5896,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="P25" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="R25" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="S25" s="68" t="n">
         <f aca="false">SUM(S9:S24)</f>
@@ -5910,15 +5972,15 @@
         <v>0</v>
       </c>
       <c r="U25" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="W25" s="55" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C26" s="71" t="n">
         <f aca="false">C25-D25</f>
@@ -5926,7 +5988,7 @@
       </c>
       <c r="D26" s="72"/>
       <c r="G26" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="H26" s="71" t="n">
         <f aca="false">H25-I25</f>
@@ -5939,7 +6001,7 @@
         <v>0</v>
       </c>
       <c r="P26" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="S26" s="73"/>
       <c r="T26" s="74" t="n">
@@ -5947,44 +6009,44 @@
         <v>0</v>
       </c>
       <c r="U26" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="W26" s="55" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="W27" s="55" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="58" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="C28" s="58"/>
       <c r="D28" s="58"/>
       <c r="E28" s="58"/>
       <c r="G28" s="58" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="H28" s="58"/>
       <c r="I28" s="58"/>
       <c r="J28" s="58"/>
       <c r="M28" s="59" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="N28" s="59"/>
       <c r="O28" s="59"/>
       <c r="P28" s="59"/>
       <c r="R28" s="59" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="S28" s="59"/>
       <c r="T28" s="59"/>
       <c r="U28" s="59"/>
       <c r="W28" s="55" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5992,10 +6054,10 @@
         <v>107</v>
       </c>
       <c r="C29" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="D29" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E29" s="60" t="s">
         <v>107</v>
@@ -6004,10 +6066,10 @@
         <v>107</v>
       </c>
       <c r="H29" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="I29" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="J29" s="60" t="s">
         <v>107</v>
@@ -6016,10 +6078,10 @@
         <v>107</v>
       </c>
       <c r="N29" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="O29" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="P29" s="60" t="s">
         <v>107</v>
@@ -6028,27 +6090,27 @@
         <v>107</v>
       </c>
       <c r="S29" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="T29" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="U29" s="60" t="s">
         <v>107</v>
       </c>
       <c r="W29" s="55" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C30" s="63"/>
       <c r="D30" s="64"/>
       <c r="E30" s="62"/>
       <c r="G30" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="H30" s="63"/>
       <c r="I30" s="64"/>
@@ -6057,16 +6119,16 @@
       <c r="N30" s="63"/>
       <c r="O30" s="64"/>
       <c r="P30" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="R30" s="62"/>
       <c r="S30" s="63"/>
       <c r="T30" s="64"/>
       <c r="U30" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="W30" s="51" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6087,7 +6149,7 @@
       <c r="T31" s="54"/>
       <c r="U31" s="65"/>
       <c r="W31" s="55" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6344,7 +6406,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C46" s="68" t="n">
         <f aca="false">SUM(C30:C45)</f>
@@ -6355,10 +6417,10 @@
         <v>0</v>
       </c>
       <c r="E46" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="G46" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="H46" s="68" t="n">
         <f aca="false">SUM(H30:H45)</f>
@@ -6369,10 +6431,10 @@
         <v>0</v>
       </c>
       <c r="J46" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="M46" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="N46" s="68" t="n">
         <f aca="false">SUM(N30:N45)</f>
@@ -6383,10 +6445,10 @@
         <v>0</v>
       </c>
       <c r="P46" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="R46" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="S46" s="68" t="n">
         <f aca="false">SUM(S30:S45)</f>
@@ -6397,12 +6459,12 @@
         <v>0</v>
       </c>
       <c r="U46" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C47" s="71" t="n">
         <f aca="false">C46-D46</f>
@@ -6410,7 +6472,7 @@
       </c>
       <c r="D47" s="72"/>
       <c r="G47" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="H47" s="71" t="n">
         <f aca="false">H46-I46</f>
@@ -6423,7 +6485,7 @@
         <v>0</v>
       </c>
       <c r="P47" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="S47" s="73"/>
       <c r="T47" s="74" t="n">
@@ -6431,30 +6493,30 @@
         <v>0</v>
       </c>
       <c r="U47" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="58" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="C49" s="58"/>
       <c r="D49" s="58"/>
       <c r="E49" s="58"/>
       <c r="G49" s="58" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="H49" s="58"/>
       <c r="I49" s="58"/>
       <c r="J49" s="58"/>
       <c r="M49" s="59" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="N49" s="59"/>
       <c r="O49" s="59"/>
       <c r="P49" s="59"/>
       <c r="R49" s="59" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="S49" s="59"/>
       <c r="T49" s="59"/>
@@ -6465,10 +6527,10 @@
         <v>107</v>
       </c>
       <c r="C50" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="D50" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E50" s="60" t="s">
         <v>107</v>
@@ -6477,10 +6539,10 @@
         <v>107</v>
       </c>
       <c r="H50" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="I50" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="J50" s="60" t="s">
         <v>107</v>
@@ -6489,10 +6551,10 @@
         <v>107</v>
       </c>
       <c r="N50" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="O50" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="P50" s="60" t="s">
         <v>107</v>
@@ -6501,10 +6563,10 @@
         <v>107</v>
       </c>
       <c r="S50" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="T50" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="U50" s="60" t="s">
         <v>107</v>
@@ -6512,13 +6574,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C51" s="63"/>
       <c r="D51" s="64"/>
       <c r="E51" s="62"/>
       <c r="G51" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="H51" s="63"/>
       <c r="I51" s="64"/>
@@ -6527,13 +6589,13 @@
       <c r="N51" s="63"/>
       <c r="O51" s="64"/>
       <c r="P51" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="R51" s="62"/>
       <c r="S51" s="63"/>
       <c r="T51" s="64"/>
       <c r="U51" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6542,7 +6604,7 @@
       <c r="D52" s="54"/>
       <c r="E52" s="65"/>
       <c r="G52" s="65" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="H52" s="66" t="n">
         <v>900000</v>
@@ -6551,7 +6613,7 @@
         <v>930000</v>
       </c>
       <c r="J52" s="65" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="M52" s="65"/>
       <c r="N52" s="66"/>
@@ -6568,7 +6630,7 @@
       <c r="D53" s="54"/>
       <c r="E53" s="65"/>
       <c r="G53" s="65" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H53" s="66" t="n">
         <v>30000</v>
@@ -6820,7 +6882,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C67" s="68" t="n">
         <f aca="false">SUM(C51:C66)</f>
@@ -6831,10 +6893,10 @@
         <v>0</v>
       </c>
       <c r="E67" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="G67" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="H67" s="68" t="n">
         <f aca="false">SUM(H51:H66)</f>
@@ -6845,10 +6907,10 @@
         <v>930000</v>
       </c>
       <c r="J67" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="M67" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="N67" s="68" t="n">
         <f aca="false">SUM(N51:N66)</f>
@@ -6859,10 +6921,10 @@
         <v>0</v>
       </c>
       <c r="P67" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="R67" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="S67" s="68" t="n">
         <f aca="false">SUM(S51:S66)</f>
@@ -6873,12 +6935,12 @@
         <v>0</v>
       </c>
       <c r="U67" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C68" s="71" t="n">
         <f aca="false">C67-D67</f>
@@ -6886,7 +6948,7 @@
       </c>
       <c r="D68" s="72"/>
       <c r="G68" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="H68" s="71" t="n">
         <f aca="false">H67-I67</f>
@@ -6899,7 +6961,7 @@
         <v>0</v>
       </c>
       <c r="P68" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="S68" s="73"/>
       <c r="T68" s="74" t="n">
@@ -6907,30 +6969,30 @@
         <v>0</v>
       </c>
       <c r="U68" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B70" s="58" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C70" s="58"/>
       <c r="D70" s="58"/>
       <c r="E70" s="58"/>
       <c r="G70" s="58" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="H70" s="58"/>
       <c r="I70" s="58"/>
       <c r="J70" s="58"/>
       <c r="M70" s="59" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="N70" s="59"/>
       <c r="O70" s="59"/>
       <c r="P70" s="59"/>
       <c r="R70" s="59" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="S70" s="59"/>
       <c r="T70" s="59"/>
@@ -6941,10 +7003,10 @@
         <v>107</v>
       </c>
       <c r="C71" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="D71" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E71" s="60" t="s">
         <v>107</v>
@@ -6953,10 +7015,10 @@
         <v>107</v>
       </c>
       <c r="H71" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="I71" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="J71" s="60" t="s">
         <v>107</v>
@@ -6965,10 +7027,10 @@
         <v>107</v>
       </c>
       <c r="N71" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="O71" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="P71" s="60" t="s">
         <v>107</v>
@@ -6977,10 +7039,10 @@
         <v>107</v>
       </c>
       <c r="S71" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="T71" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="U71" s="60" t="s">
         <v>107</v>
@@ -6988,7 +7050,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C72" s="63" t="n">
         <v>5000000</v>
@@ -6996,7 +7058,7 @@
       <c r="D72" s="64"/>
       <c r="E72" s="62"/>
       <c r="G72" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="H72" s="63"/>
       <c r="I72" s="64"/>
@@ -7005,13 +7067,13 @@
       <c r="N72" s="63"/>
       <c r="O72" s="64"/>
       <c r="P72" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="R72" s="62"/>
       <c r="S72" s="63"/>
       <c r="T72" s="64"/>
       <c r="U72" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7028,7 +7090,7 @@
         <v>116</v>
       </c>
       <c r="G73" s="65" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="H73" s="66" t="n">
         <v>420000</v>
@@ -7306,7 +7368,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C88" s="68" t="n">
         <f aca="false">SUM(C72:C87)</f>
@@ -7317,10 +7379,10 @@
         <v>5000000</v>
       </c>
       <c r="E88" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="G88" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="H88" s="68" t="n">
         <f aca="false">SUM(H72:H87)</f>
@@ -7331,10 +7393,10 @@
         <v>0</v>
       </c>
       <c r="J88" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="M88" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="N88" s="68" t="n">
         <f aca="false">SUM(N72:N87)</f>
@@ -7345,10 +7407,10 @@
         <v>0</v>
       </c>
       <c r="P88" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="R88" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="S88" s="68" t="n">
         <f aca="false">SUM(S72:S87)</f>
@@ -7359,12 +7421,12 @@
         <v>750000</v>
       </c>
       <c r="U88" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C89" s="71" t="n">
         <f aca="false">C88-D88</f>
@@ -7372,7 +7434,7 @@
       </c>
       <c r="D89" s="72"/>
       <c r="G89" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="H89" s="71" t="n">
         <f aca="false">H88-I88</f>
@@ -7385,7 +7447,7 @@
         <v>0</v>
       </c>
       <c r="P89" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="S89" s="73"/>
       <c r="T89" s="74" t="n">
@@ -7393,30 +7455,30 @@
         <v>750000</v>
       </c>
       <c r="U89" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B91" s="58" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C91" s="58"/>
       <c r="D91" s="58"/>
       <c r="E91" s="58"/>
       <c r="G91" s="58" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="H91" s="58"/>
       <c r="I91" s="58"/>
       <c r="J91" s="58"/>
       <c r="M91" s="59" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="N91" s="59"/>
       <c r="O91" s="59"/>
       <c r="P91" s="59"/>
       <c r="R91" s="59" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="S91" s="59"/>
       <c r="T91" s="59"/>
@@ -7427,10 +7489,10 @@
         <v>107</v>
       </c>
       <c r="C92" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="D92" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E92" s="60" t="s">
         <v>107</v>
@@ -7439,10 +7501,10 @@
         <v>107</v>
       </c>
       <c r="H92" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="I92" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="J92" s="60" t="s">
         <v>107</v>
@@ -7451,10 +7513,10 @@
         <v>107</v>
       </c>
       <c r="N92" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="O92" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="P92" s="60" t="s">
         <v>107</v>
@@ -7463,10 +7525,10 @@
         <v>107</v>
       </c>
       <c r="S92" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="T92" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="U92" s="60" t="s">
         <v>107</v>
@@ -7474,7 +7536,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B93" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C93" s="63" t="n">
         <v>6000000</v>
@@ -7487,27 +7549,27 @@
         <v>5400000</v>
       </c>
       <c r="J93" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="M93" s="62"/>
       <c r="N93" s="63"/>
       <c r="O93" s="64"/>
       <c r="P93" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="R93" s="62"/>
       <c r="S93" s="63"/>
       <c r="T93" s="64"/>
       <c r="U93" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B94" s="65" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C94" s="66" t="n">
-        <v>630000</v>
+        <v>620000</v>
       </c>
       <c r="D94" s="54" t="n">
         <v>6000000</v>
@@ -7522,13 +7584,13 @@
         <v>5400000</v>
       </c>
       <c r="I94" s="54" t="n">
-        <v>31500</v>
+        <v>31000</v>
       </c>
       <c r="J94" s="65" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="M94" s="65" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="N94" s="66" t="n">
         <v>30000</v>
@@ -7537,7 +7599,7 @@
         <v>600000</v>
       </c>
       <c r="P94" s="65" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="R94" s="65"/>
       <c r="S94" s="66"/>
@@ -7552,13 +7614,13 @@
       <c r="G95" s="65"/>
       <c r="H95" s="66"/>
       <c r="I95" s="54" t="n">
-        <v>31500</v>
+        <v>31000</v>
       </c>
       <c r="J95" s="65" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="M95" s="65" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="N95" s="66" t="n">
         <v>30000</v>
@@ -7580,7 +7642,7 @@
       <c r="I96" s="54"/>
       <c r="J96" s="65"/>
       <c r="M96" s="65" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="N96" s="66" t="n">
         <v>30000</v>
@@ -7810,21 +7872,21 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B109" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C109" s="68" t="n">
         <f aca="false">SUM(C93:C108)</f>
-        <v>6630000</v>
+        <v>6620000</v>
       </c>
       <c r="D109" s="69" t="n">
         <f aca="false">SUM(D93:D108)</f>
         <v>6000000</v>
       </c>
       <c r="E109" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="G109" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="H109" s="68" t="n">
         <f aca="false">SUM(H93:H108)</f>
@@ -7832,13 +7894,13 @@
       </c>
       <c r="I109" s="69" t="n">
         <f aca="false">SUM(I93:I108)</f>
-        <v>5463000</v>
+        <v>5462000</v>
       </c>
       <c r="J109" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="M109" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="N109" s="68" t="n">
         <f aca="false">SUM(N93:N108)</f>
@@ -7849,10 +7911,10 @@
         <v>600000</v>
       </c>
       <c r="P109" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="R109" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="S109" s="68" t="n">
         <f aca="false">SUM(S93:S108)</f>
@@ -7863,25 +7925,25 @@
         <v>0</v>
       </c>
       <c r="U109" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B110" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C110" s="71" t="n">
         <f aca="false">C109-D109</f>
-        <v>630000</v>
+        <v>620000</v>
       </c>
       <c r="D110" s="72"/>
       <c r="H110" s="73"/>
       <c r="I110" s="76" t="n">
         <f aca="false">I109-H109</f>
-        <v>63000</v>
+        <v>62000</v>
       </c>
       <c r="J110" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="N110" s="73"/>
       <c r="O110" s="74" t="n">
@@ -7889,7 +7951,7 @@
         <v>510000</v>
       </c>
       <c r="P110" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="S110" s="73"/>
       <c r="T110" s="74" t="n">
@@ -7897,30 +7959,30 @@
         <v>0</v>
       </c>
       <c r="U110" s="75" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B112" s="58" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C112" s="58"/>
       <c r="D112" s="58"/>
       <c r="E112" s="58"/>
       <c r="G112" s="58" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="H112" s="58"/>
       <c r="I112" s="58"/>
       <c r="J112" s="58"/>
       <c r="M112" s="77" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="N112" s="77"/>
       <c r="O112" s="77"/>
       <c r="P112" s="77"/>
       <c r="R112" s="77" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="S112" s="77"/>
       <c r="T112" s="77"/>
@@ -7931,10 +7993,10 @@
         <v>107</v>
       </c>
       <c r="C113" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="D113" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E113" s="60" t="s">
         <v>107</v>
@@ -7943,10 +8005,10 @@
         <v>107</v>
       </c>
       <c r="H113" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="I113" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="J113" s="60" t="s">
         <v>107</v>
@@ -7955,10 +8017,10 @@
         <v>107</v>
       </c>
       <c r="N113" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="O113" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="P113" s="60" t="s">
         <v>107</v>
@@ -7967,10 +8029,10 @@
         <v>107</v>
       </c>
       <c r="S113" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="T113" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="U113" s="60" t="s">
         <v>107</v>
@@ -7978,7 +8040,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B114" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C114" s="63"/>
       <c r="D114" s="64"/>
@@ -7987,37 +8049,37 @@
       <c r="H114" s="63"/>
       <c r="I114" s="64"/>
       <c r="J114" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="M114" s="62"/>
       <c r="N114" s="63"/>
       <c r="O114" s="64"/>
       <c r="P114" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="R114" s="62"/>
       <c r="S114" s="63"/>
       <c r="T114" s="64"/>
       <c r="U114" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B115" s="65" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C115" s="66" t="n">
-        <v>300000</v>
+        <v>310000</v>
       </c>
       <c r="D115" s="54"/>
       <c r="E115" s="65"/>
       <c r="G115" s="65"/>
       <c r="H115" s="66"/>
       <c r="I115" s="54" t="n">
-        <v>30000</v>
+        <v>31000</v>
       </c>
       <c r="J115" s="65" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="M115" s="65"/>
       <c r="N115" s="66"/>
@@ -8040,10 +8102,10 @@
       <c r="G116" s="65"/>
       <c r="H116" s="66"/>
       <c r="I116" s="54" t="n">
-        <v>34000</v>
+        <v>35000</v>
       </c>
       <c r="J116" s="65" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="M116" s="65"/>
       <c r="N116" s="66"/>
@@ -8056,7 +8118,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B117" s="65" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C117" s="66" t="n">
         <v>196600</v>
@@ -8078,10 +8140,10 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B118" s="65" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C118" s="66" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="D118" s="54"/>
       <c r="E118" s="65"/>
@@ -8298,21 +8360,21 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B130" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C130" s="68" t="n">
         <f aca="false">SUM(C114:C129)</f>
-        <v>538600</v>
+        <v>549600</v>
       </c>
       <c r="D130" s="69" t="n">
         <f aca="false">SUM(D114:D129)</f>
         <v>0</v>
       </c>
       <c r="E130" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="G130" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="H130" s="68" t="n">
         <f aca="false">SUM(H114:H129)</f>
@@ -8320,13 +8382,13 @@
       </c>
       <c r="I130" s="69" t="n">
         <f aca="false">SUM(I114:I129)</f>
-        <v>64000</v>
+        <v>66000</v>
       </c>
       <c r="J130" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="M130" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="N130" s="68" t="n">
         <f aca="false">SUM(N114:N129)</f>
@@ -8337,10 +8399,10 @@
         <v>0</v>
       </c>
       <c r="P130" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="R130" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="S130" s="68" t="n">
         <f aca="false">SUM(S114:S129)</f>
@@ -8351,25 +8413,25 @@
         <v>0</v>
       </c>
       <c r="U130" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B131" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C131" s="71" t="n">
         <f aca="false">C130-D130</f>
-        <v>538600</v>
+        <v>549600</v>
       </c>
       <c r="D131" s="72"/>
       <c r="H131" s="73"/>
       <c r="I131" s="76" t="n">
         <f aca="false">I130-H130</f>
-        <v>64000</v>
+        <v>66000</v>
       </c>
       <c r="J131" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="N131" s="73"/>
       <c r="O131" s="78" t="n">
@@ -8377,7 +8439,7 @@
         <v>0</v>
       </c>
       <c r="P131" s="79" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="S131" s="73"/>
       <c r="T131" s="78" t="n">
@@ -8385,30 +8447,30 @@
         <v>0</v>
       </c>
       <c r="U131" s="79" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B133" s="58" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C133" s="58"/>
       <c r="D133" s="58"/>
       <c r="E133" s="58"/>
       <c r="G133" s="58" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="H133" s="58"/>
       <c r="I133" s="58"/>
       <c r="J133" s="58"/>
       <c r="M133" s="77" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="N133" s="77"/>
       <c r="O133" s="77"/>
       <c r="P133" s="77"/>
       <c r="R133" s="80" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="S133" s="80"/>
       <c r="T133" s="80"/>
@@ -8419,10 +8481,10 @@
         <v>107</v>
       </c>
       <c r="C134" s="61" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="D134" s="60" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E134" s="60" t="s">
         <v>107</v>
@@ -8431,10 +8493,10 @@
         <v>107</v>
       </c>
       <c r="H134" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="I134" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="J134" s="60" t="s">
         <v>107</v>
@@ -8443,10 +8505,10 @@
         <v>107</v>
       </c>
       <c r="N134" s="61" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="O134" s="60" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="P134" s="60" t="s">
         <v>107</v>
@@ -8455,10 +8517,10 @@
         <v>107</v>
       </c>
       <c r="S134" s="61" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="T134" s="60" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="U134" s="60" t="s">
         <v>107</v>
@@ -8466,7 +8528,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B135" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C135" s="63"/>
       <c r="D135" s="64"/>
@@ -8475,24 +8537,24 @@
       <c r="H135" s="63"/>
       <c r="I135" s="64"/>
       <c r="J135" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="M135" s="62"/>
       <c r="N135" s="63"/>
       <c r="O135" s="64"/>
       <c r="P135" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="R135" s="62"/>
       <c r="S135" s="63"/>
       <c r="T135" s="64"/>
       <c r="U135" s="62" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B136" s="65" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C136" s="66" t="n">
         <v>1000000</v>
@@ -8502,10 +8564,10 @@
       <c r="G136" s="65"/>
       <c r="H136" s="66"/>
       <c r="I136" s="54" t="n">
-        <v>23667</v>
+        <v>142000</v>
       </c>
       <c r="J136" s="65" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="M136" s="65"/>
       <c r="N136" s="66"/>
@@ -8532,7 +8594,7 @@
       <c r="G137" s="65"/>
       <c r="H137" s="66"/>
       <c r="I137" s="54" t="n">
-        <v>396333</v>
+        <v>278000</v>
       </c>
       <c r="J137" s="65" t="s">
         <v>152</v>
@@ -8542,16 +8604,16 @@
       <c r="O137" s="54"/>
       <c r="P137" s="65"/>
       <c r="R137" s="65" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="S137" s="66" t="n">
         <v>28500</v>
       </c>
       <c r="T137" s="54" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="U137" s="65" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8568,16 +8630,16 @@
       <c r="O138" s="54"/>
       <c r="P138" s="65"/>
       <c r="R138" s="65" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="S138" s="66" t="n">
-        <v>61500</v>
+        <v>62000</v>
       </c>
       <c r="T138" s="54" t="n">
         <v>420000</v>
       </c>
       <c r="U138" s="65" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8616,7 +8678,7 @@
       <c r="O140" s="54"/>
       <c r="P140" s="65"/>
       <c r="R140" s="65" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="S140" s="66" t="n">
         <v>27000</v>
@@ -8638,10 +8700,10 @@
       <c r="O141" s="54"/>
       <c r="P141" s="65"/>
       <c r="R141" s="65" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="S141" s="66" t="n">
-        <v>23667</v>
+        <v>142000</v>
       </c>
       <c r="T141" s="54"/>
       <c r="U141" s="65"/>
@@ -8663,7 +8725,7 @@
         <v>152</v>
       </c>
       <c r="S142" s="66" t="n">
-        <v>396333</v>
+        <v>278000</v>
       </c>
       <c r="T142" s="54"/>
       <c r="U142" s="65"/>
@@ -8682,10 +8744,10 @@
       <c r="O143" s="54"/>
       <c r="P143" s="65"/>
       <c r="R143" s="65" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="S143" s="66" t="n">
-        <v>65500</v>
+        <v>66000</v>
       </c>
       <c r="T143" s="54"/>
       <c r="U143" s="65"/>
@@ -8818,7 +8880,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B151" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C151" s="68" t="n">
         <f aca="false">SUM(C135:C150)</f>
@@ -8829,10 +8891,10 @@
         <v>0</v>
       </c>
       <c r="E151" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="G151" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="H151" s="68" t="n">
         <f aca="false">SUM(H135:H150)</f>
@@ -8843,10 +8905,10 @@
         <v>420000</v>
       </c>
       <c r="J151" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="M151" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="N151" s="68" t="n">
         <f aca="false">SUM(N135:N150)</f>
@@ -8857,26 +8919,26 @@
         <v>0</v>
       </c>
       <c r="P151" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="R151" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="S151" s="68" t="n">
         <f aca="false">SUM(S135:S150)</f>
-        <v>834500</v>
+        <v>835500</v>
       </c>
       <c r="T151" s="69" t="n">
         <f aca="false">SUM(T135:T150)</f>
-        <v>7822000</v>
+        <v>7823000</v>
       </c>
       <c r="U151" s="67" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B152" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C152" s="71" t="n">
         <f aca="false">C151-D151</f>
@@ -8889,7 +8951,7 @@
         <v>420000</v>
       </c>
       <c r="J152" s="70" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="N152" s="73"/>
       <c r="O152" s="78" t="n">
@@ -8897,7 +8959,7 @@
         <v>0</v>
       </c>
       <c r="P152" s="79" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="S152" s="73"/>
       <c r="T152" s="81" t="n">
@@ -8905,12 +8967,12 @@
         <v>6987500</v>
       </c>
       <c r="U152" s="82" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B155" s="83" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="C155" s="83"/>
       <c r="D155" s="83"/>
@@ -8922,14 +8984,14 @@
       <c r="J155" s="83"/>
       <c r="L155" s="84" t="n">
         <f aca="false">(C25+H25+C46+H46+C67+H67+C88+H88+C109+H109+C130+H130+C151+H151+N25+S25+N46+S46+N67+S67+N88+S88+N109+S109+N130+S130+N151+S151)-(C9+H9+C30+H30+C51+H51+C72+H72+C93+H93+C114+H114+C135+H135+N9+S9+N30+S30+N51+S51+N72+S72+N93+S93+N114+S114+N135+S135)</f>
-        <v>24318100</v>
+        <v>24320100</v>
       </c>
       <c r="M155" s="84"/>
       <c r="N155" s="84"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B156" s="83" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="C156" s="83"/>
       <c r="D156" s="83"/>
@@ -8941,14 +9003,14 @@
       <c r="J156" s="83"/>
       <c r="L156" s="84" t="n">
         <f aca="false">(D25+I25+D46+I46+D67+I67+D88+I88+D109+I109+D130+I130+D151+I151+O25+T25+O46+T46+O67+T67+O88+T88+O109+T109+O130+T130+O151+T151)-(D9+I9+D30+I30+D51+I51+D72+I72+D93+I93+D114+I114+D135+I135+O9+T9+O30+T30+O51+T51+O72+T72+O93+T93+O114+T114+O135+T135)</f>
-        <v>24318100</v>
+        <v>24320100</v>
       </c>
       <c r="M156" s="84"/>
       <c r="N156" s="84"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B157" s="83" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="C157" s="83"/>
       <c r="D157" s="83"/>
@@ -9042,7 +9104,7 @@
         <v>69</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9051,10 +9113,10 @@
         <v>Marketable securities</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9066,7 +9128,7 @@
         <v>72</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9075,10 +9137,10 @@
         <v>Inventories</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9087,7 +9149,7 @@
         <v>Prepaid rent / prepaid expenses</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9096,7 +9158,7 @@
         <v>Construction in progress (2019)</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9105,7 +9167,7 @@
         <v>Land</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9114,7 +9176,7 @@
         <v>Development costs – Baldnessox</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9123,7 +9185,7 @@
         <v>Buildings (old premises + new building)</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9132,7 +9194,7 @@
         <v>Accum. depreciation – Buildings</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>